<commit_message>
Add profitable utilization scenario
</commit_message>
<xml_diff>
--- a/eride_operating_model.xlsx
+++ b/eride_operating_model.xlsx
@@ -2,35 +2,63 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="600" firstSheet="0" activeTab="4" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inputs" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Model" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cost_Breakdown" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cloud_Tiers" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dev_Budget" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scenario_Comparison" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Model" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cost_Breakdown" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cloud_Tiers" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dev_Budget" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1" forceFullCalc="1"/>
+  <calcPr calcId="191029" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="0.0%"/>
+    <numFmt numFmtId="165" formatCode="_-[$PHP]\ * #,##0.00_-;\-[$PHP]\ * #,##0.00_-;_-[$PHP]\ * &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="166" formatCode="0.0x"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <b val="1"/>
+      <color rgb="FF142334"/>
+      <sz val="18"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <color rgb="FF607386"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <b val="1"/>
+      <sz val="11"/>
     </font>
     <font>
       <b val="1"/>
@@ -45,11 +73,8 @@
       <b val="1"/>
       <color rgb="00FFFFFF"/>
     </font>
-    <font>
-      <b val="1"/>
-    </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -58,7 +83,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF6E5"/>
+        <fgColor rgb="FFFFF6E5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF142334"/>
       </patternFill>
     </fill>
     <fill>
@@ -67,12 +97,27 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFDCE5ED"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFDCE5ED"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFDCE5ED"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFDCE5ED"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -93,7 +138,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -122,9 +167,42 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -210,7 +288,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>Monthly cost breakdown</a:t>
+              <a:t>Monthly profit/loss by scenario</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -225,7 +303,7 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'Cost_Breakdown'!B4</f>
+              <f>'Scenario_Comparison'!J4</f>
             </strRef>
           </tx>
           <spPr>
@@ -235,12 +313,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Cost_Breakdown'!$A$5:$A$15</f>
+              <f>'Scenario_Comparison'!$A$5:$A$6</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Cost_Breakdown'!$B$5:$B$15</f>
+              <f>'Scenario_Comparison'!$J$5:$J$6</f>
             </numRef>
           </val>
         </ser>
@@ -302,26 +380,243 @@
       <tx>
         <rich>
           <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
           <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
             <a:r>
+              <a:rPr lang="en-GB"/>
+              <a:t>Monthly cost breakdown</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+      <overlay val="1"/>
+    </title>
+    <plotArea>
+      <layout/>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <varyColors val="1"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>Cost_Breakdown!$B$4</f>
+              <strCache>
+                <ptCount val="1"/>
+                <pt idx="0">
+                  <v>Monthly PHP</v>
+                </pt>
+              </strCache>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <invertIfNegative val="1"/>
+          <cat>
+            <strRef>
+              <f>Cost_Breakdown!$A$5:$A$15</f>
+              <strCache>
+                <ptCount val="11"/>
+                <pt idx="0">
+                  <v>Rider base payroll</v>
+                </pt>
+                <pt idx="1">
+                  <v>Rider incentives</v>
+                </pt>
+                <pt idx="2">
+                  <v>Electricity</v>
+                </pt>
+                <pt idx="3">
+                  <v>Fleet acquisition / amortization</v>
+                </pt>
+                <pt idx="4">
+                  <v>Fleet maintenance, insurance, registration</v>
+                </pt>
+                <pt idx="5">
+                  <v>Development build recovery</v>
+                </pt>
+                <pt idx="6">
+                  <v>Ongoing dev support retainer</v>
+                </pt>
+                <pt idx="7">
+                  <v>Cloud / API cost</v>
+                </pt>
+                <pt idx="8">
+                  <v>Operations, support and admin</v>
+                </pt>
+                <pt idx="9">
+                  <v>Payment processing</v>
+                </pt>
+                <pt idx="10">
+                  <v>Tax / regulatory reserve</v>
+                </pt>
+              </strCache>
+            </strRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>Cost_Breakdown!$B$5:$B$15</f>
+              <numCache>
+                <formatCode>#,##0.00</formatCode>
+                <ptCount val="11"/>
+                <pt idx="0">
+                  <v>1039025</v>
+                </pt>
+                <pt idx="1">
+                  <v>0</v>
+                </pt>
+                <pt idx="2">
+                  <v>41067</v>
+                </pt>
+                <pt idx="3">
+                  <v>104166.6666666667</v>
+                </pt>
+                <pt idx="4">
+                  <v>100000</v>
+                </pt>
+                <pt idx="5">
+                  <v>166666.6666666667</v>
+                </pt>
+                <pt idx="6">
+                  <v>55000</v>
+                </pt>
+                <pt idx="7">
+                  <v>38843.3</v>
+                </pt>
+                <pt idx="8">
+                  <v>146250</v>
+                </pt>
+                <pt idx="9">
+                  <v>9674.4375</v>
+                </pt>
+                <pt idx="10">
+                  <v>33169.5</v>
+                </pt>
+              </numCache>
+            </numRef>
+          </val>
+        </ser>
+        <dLbls>
+          <showLegendKey val="0"/>
+          <showVal val="0"/>
+          <showCatName val="0"/>
+          <showSerName val="0"/>
+          <showPercent val="0"/>
+          <showBubbleSize val="0"/>
+        </dLbls>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <delete val="1"/>
+        <axPos val="b"/>
+        <numFmt formatCode="General" sourceLinked="1"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <tickLblPos val="nextTo"/>
+        <crossAx val="100"/>
+        <crosses val="autoZero"/>
+        <auto val="1"/>
+        <lblAlgn val="ctr"/>
+        <lblOffset val="100"/>
+        <noMultiLvlLbl val="1"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <delete val="1"/>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-GB"/>
+                  <a:t>PHP/month</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+          <overlay val="1"/>
+        </title>
+        <numFmt formatCode="#,##0.00" sourceLinked="1"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <tickLblPos val="nextTo"/>
+        <crossAx val="10"/>
+        <crosses val="autoZero"/>
+        <crossBetween val="between"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+      <overlay val="0"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-GB"/>
               <a:t>Cloud/API cost by user tier</a:t>
             </a:r>
           </a:p>
         </rich>
       </tx>
+      <overlay val="1"/>
     </title>
     <plotArea>
+      <layout/>
       <lineChart>
         <grouping val="standard"/>
+        <varyColors val="1"/>
         <ser>
           <idx val="0"/>
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'Cloud_Tiers'!B4</f>
+              <f>Cloud_Tiers!$B$4</f>
+              <strCache>
+                <ptCount val="1"/>
+                <pt idx="0">
+                  <v>Estimated monthly cloud/API cost</v>
+                </pt>
+              </strCache>
             </strRef>
           </tx>
           <spPr>
@@ -339,15 +634,81 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Cloud_Tiers'!$C$5:$C$12</f>
+              <f>Cloud_Tiers!$C$5:$C$12</f>
+              <numCache>
+                <formatCode>#,##0</formatCode>
+                <ptCount val="8"/>
+                <pt idx="0">
+                  <v>20</v>
+                </pt>
+                <pt idx="1">
+                  <v>100</v>
+                </pt>
+                <pt idx="2">
+                  <v>500</v>
+                </pt>
+                <pt idx="3">
+                  <v>1000</v>
+                </pt>
+                <pt idx="4">
+                  <v>3750</v>
+                </pt>
+                <pt idx="5">
+                  <v>5000</v>
+                </pt>
+                <pt idx="6">
+                  <v>10000</v>
+                </pt>
+                <pt idx="7">
+                  <v>25000</v>
+                </pt>
+              </numCache>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Cloud_Tiers'!$B$5:$B$12</f>
+              <f>Cloud_Tiers!$B$5:$B$12</f>
+              <numCache>
+                <formatCode>#,##0.00</formatCode>
+                <ptCount val="8"/>
+                <pt idx="0">
+                  <v>1500</v>
+                </pt>
+                <pt idx="1">
+                  <v>1582.07</v>
+                </pt>
+                <pt idx="2">
+                  <v>15000.95</v>
+                </pt>
+                <pt idx="3">
+                  <v>38843.3</v>
+                </pt>
+                <pt idx="4">
+                  <v>169976.225</v>
+                </pt>
+                <pt idx="5">
+                  <v>229582.1</v>
+                </pt>
+                <pt idx="6">
+                  <v>468005.6</v>
+                </pt>
+                <pt idx="7">
+                  <v>1183276.1</v>
+                </pt>
+              </numCache>
             </numRef>
           </val>
+          <smooth val="1"/>
         </ser>
+        <dLbls>
+          <showLegendKey val="0"/>
+          <showVal val="0"/>
+          <showCatName val="0"/>
+          <showSerName val="0"/>
+          <showPercent val="0"/>
+          <showBubbleSize val="0"/>
+        </dLbls>
+        <smooth val="0"/>
         <axId val="10"/>
         <axId val="100"/>
       </lineChart>
@@ -356,26 +717,39 @@
         <scaling>
           <orientation val="minMax"/>
         </scaling>
-        <axPos val="l"/>
+        <delete val="1"/>
+        <axPos val="b"/>
+        <numFmt formatCode="#,##0" sourceLinked="1"/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
+        <tickLblPos val="nextTo"/>
         <crossAx val="100"/>
+        <crosses val="autoZero"/>
+        <auto val="1"/>
+        <lblAlgn val="ctr"/>
         <lblOffset val="100"/>
+        <noMultiLvlLbl val="1"/>
       </catAx>
       <valAx>
         <axId val="100"/>
         <scaling>
           <orientation val="minMax"/>
         </scaling>
+        <delete val="1"/>
         <axPos val="l"/>
         <majorGridlines/>
+        <numFmt formatCode="#,##0.00" sourceLinked="1"/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
+        <tickLblPos val="nextTo"/>
         <crossAx val="10"/>
+        <crosses val="autoZero"/>
+        <crossBetween val="between"/>
       </valAx>
     </plotArea>
     <legend>
       <legendPos val="r"/>
+      <overlay val="0"/>
     </legend>
     <plotVisOnly val="1"/>
     <dispBlanksAs val="gap"/>
@@ -384,6 +758,33 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>11</col>
+      <colOff>0</colOff>
+      <row>3</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5040000" cy="2520000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
@@ -410,7 +811,7 @@
 </wsDr>
 </file>
 
-<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
@@ -727,7 +1128,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:D46"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
@@ -735,7 +1136,7 @@
     <col width="48" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="23.4" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>E-Ride Operating Model - Inputs</t>
@@ -1634,821 +2035,202 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D40"/>
+  <dimension ref="A1:J6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="34" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="24" customWidth="1" min="3" max="3"/>
-    <col width="48" customWidth="1" min="4" max="4"/>
+    <col width="32" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>E-Ride Operating Model - Calculations</t>
-        </is>
-      </c>
-      <c r="B1" s="2" t="n"/>
-      <c r="C1" s="2" t="n"/>
-      <c r="D1" s="2" t="n"/>
+      <c r="A1" s="12" t="inlineStr">
+        <is>
+          <t>Scenario Comparison - Wage Coverage and Profitability</t>
+        </is>
+      </c>
+      <c r="B1" s="13" t="n"/>
+      <c r="C1" s="13" t="n"/>
+      <c r="D1" s="13" t="n"/>
+      <c r="E1" s="13" t="n"/>
+      <c r="F1" s="13" t="n"/>
+      <c r="G1" s="13" t="n"/>
+      <c r="H1" s="13" t="n"/>
+      <c r="I1" s="13" t="n"/>
+      <c r="J1" s="13" t="n"/>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="inlineStr">
-        <is>
-          <t>Core deterministic calculation. This is the Excel fallback for the dashboard.</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="n"/>
-      <c r="C2" s="2" t="n"/>
-      <c r="D2" s="2" t="n"/>
+      <c r="A2" s="14" t="inlineStr">
+        <is>
+          <t>Current setup versus a profitable utilization case that generates fare revenue well above rider wage cost.</t>
+        </is>
+      </c>
+      <c r="B2" s="13" t="n"/>
+      <c r="C2" s="13" t="n"/>
+      <c r="D2" s="13" t="n"/>
+      <c r="E2" s="13" t="n"/>
+      <c r="F2" s="13" t="n"/>
+      <c r="G2" s="13" t="n"/>
+      <c r="H2" s="13" t="n"/>
+      <c r="I2" s="13" t="n"/>
+      <c r="J2" s="13" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="n"/>
-      <c r="B3" s="2" t="n"/>
-      <c r="C3" s="2" t="n"/>
-      <c r="D3" s="2" t="n"/>
+      <c r="A3" s="13" t="n"/>
+      <c r="B3" s="13" t="n"/>
+      <c r="C3" s="13" t="n"/>
+      <c r="D3" s="13" t="n"/>
+      <c r="E3" s="13" t="n"/>
+      <c r="F3" s="13" t="n"/>
+      <c r="G3" s="13" t="n"/>
+      <c r="H3" s="13" t="n"/>
+      <c r="I3" s="13" t="n"/>
+      <c r="J3" s="13" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>Metric</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>Formula / Value</t>
-        </is>
-      </c>
-      <c r="C4" s="4" t="inlineStr">
-        <is>
-          <t>Unit</t>
-        </is>
-      </c>
-      <c r="D4" s="4" t="inlineStr">
-        <is>
-          <t>Meaning</t>
+      <c r="A4" s="15" t="inlineStr">
+        <is>
+          <t>Scenario</t>
+        </is>
+      </c>
+      <c r="B4" s="15" t="inlineStr">
+        <is>
+          <t>Active users</t>
+        </is>
+      </c>
+      <c r="C4" s="15" t="inlineStr">
+        <is>
+          <t>Riders</t>
+        </is>
+      </c>
+      <c r="D4" s="15" t="inlineStr">
+        <is>
+          <t>Rides/user/month</t>
+        </is>
+      </c>
+      <c r="E4" s="15" t="inlineStr">
+        <is>
+          <t>Requested rides/rider/day</t>
+        </is>
+      </c>
+      <c r="F4" s="15" t="inlineStr">
+        <is>
+          <t>Completed rides/rider/day</t>
+        </is>
+      </c>
+      <c r="G4" s="15" t="inlineStr">
+        <is>
+          <t>Fare revenue/rider/day</t>
+        </is>
+      </c>
+      <c r="H4" s="15" t="inlineStr">
+        <is>
+          <t>Wage cost/rider/day</t>
+        </is>
+      </c>
+      <c r="I4" s="15" t="inlineStr">
+        <is>
+          <t>Wage coverage</t>
+        </is>
+      </c>
+      <c r="J4" s="15" t="inlineStr">
+        <is>
+          <t>Monthly profit/loss</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>Short distance km</t>
-        </is>
-      </c>
-      <c r="B5" s="6">
-        <f>MIN(MAX(Inputs!B14-Inputs!B17,0),MAX(Inputs!B19-Inputs!B17,0))</f>
-        <v/>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>km</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>Charged at regular per-km rate</t>
-        </is>
+      <c r="A5" s="13" t="inlineStr">
+        <is>
+          <t>Current setup</t>
+        </is>
+      </c>
+      <c r="B5" s="16">
+        <f>Inputs!B8</f>
+        <v/>
+      </c>
+      <c r="C5" s="16">
+        <f>Inputs!B9</f>
+        <v/>
+      </c>
+      <c r="D5" s="17">
+        <f>Inputs!B10</f>
+        <v/>
+      </c>
+      <c r="E5" s="17">
+        <f>Inputs!B11</f>
+        <v/>
+      </c>
+      <c r="F5" s="17">
+        <f>Model!B15</f>
+        <v/>
+      </c>
+      <c r="G5" s="17">
+        <f>Model!B20</f>
+        <v/>
+      </c>
+      <c r="H5" s="17">
+        <f>Inputs!B26*(1+Inputs!B27)</f>
+        <v/>
+      </c>
+      <c r="I5" s="18">
+        <f>G5/H5</f>
+        <v/>
+      </c>
+      <c r="J5" s="17">
+        <f>Model!B32</f>
+        <v/>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>Long distance km</t>
-        </is>
-      </c>
-      <c r="B6" s="6">
-        <f>MAX(Inputs!B14-Inputs!B19,0)</f>
-        <v/>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>km</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>Charged at long-distance rate</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>Charged minutes</t>
-        </is>
-      </c>
-      <c r="B7" s="6">
-        <f>MAX(Inputs!B15-Inputs!B21,0)</f>
-        <v/>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>minutes</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>Charged beyond base minutes</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>Fare before discount</t>
-        </is>
-      </c>
-      <c r="B8" s="6">
-        <f>Inputs!B16+B5*Inputs!B18+B6*Inputs!B20+B7*Inputs!B22</f>
-        <v/>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>PHP/ride</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>Benchmark fare</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>Final passenger fare</t>
-        </is>
-      </c>
-      <c r="B9" s="6">
-        <f>B8*(1-Inputs!B23)</f>
-        <v/>
-      </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>PHP/ride</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>Passenger fare</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>Requested demand</t>
-        </is>
-      </c>
-      <c r="B10" s="6">
-        <f>Inputs!B8*Inputs!B10</f>
-        <v/>
-      </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>rides/month</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>User demand</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>Requested fleet capacity</t>
-        </is>
-      </c>
-      <c r="B11" s="6">
-        <f>Inputs!B9*Inputs!B11*Inputs!B12</f>
-        <v/>
-      </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>rides/month</t>
-        </is>
-      </c>
-      <c r="D11" s="2" t="inlineStr">
-        <is>
-          <t>Fleet capacity</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>Requested served rides</t>
-        </is>
-      </c>
-      <c r="B12" s="6">
-        <f>MIN(B10,B11)</f>
-        <v/>
-      </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>rides/month</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>Matched rides</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>Completed rides</t>
-        </is>
-      </c>
-      <c r="B13" s="6">
-        <f>B12*Inputs!B13</f>
-        <v/>
-      </c>
-      <c r="C13" s="2" t="inlineStr">
-        <is>
-          <t>rides/month</t>
-        </is>
-      </c>
-      <c r="D13" s="2" t="inlineStr">
-        <is>
-          <t>Revenue-generating rides</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>Completed rides / day</t>
-        </is>
-      </c>
-      <c r="B14" s="6">
-        <f>B13/Inputs!B12</f>
-        <v/>
-      </c>
-      <c r="C14" s="2" t="inlineStr">
-        <is>
-          <t>rides/day</t>
-        </is>
-      </c>
-      <c r="D14" s="2" t="inlineStr">
-        <is>
-          <t>Daily completed rides</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>Completed rides / rider / day</t>
-        </is>
-      </c>
-      <c r="B15" s="6">
-        <f>B13/(Inputs!B9*Inputs!B12)</f>
-        <v/>
-      </c>
-      <c r="C15" s="2" t="inlineStr">
-        <is>
-          <t>rides/rider/day</t>
-        </is>
-      </c>
-      <c r="D15" s="2" t="inlineStr">
-        <is>
-          <t>Actual utilization</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>Fare revenue</t>
-        </is>
-      </c>
-      <c r="B16" s="6">
-        <f>B13*B9*Inputs!B24</f>
-        <v/>
-      </c>
-      <c r="C16" s="2" t="inlineStr">
-        <is>
-          <t>PHP/month</t>
-        </is>
-      </c>
-      <c r="D16" s="2" t="inlineStr">
-        <is>
-          <t>Retained fare revenue</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t>Membership revenue</t>
-        </is>
-      </c>
-      <c r="B17" s="6">
-        <f>Inputs!B8*Inputs!B25</f>
-        <v/>
-      </c>
-      <c r="C17" s="2" t="inlineStr">
-        <is>
-          <t>PHP/month</t>
-        </is>
-      </c>
-      <c r="D17" s="2" t="inlineStr">
-        <is>
-          <t>Optional user fees</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>Total revenue</t>
-        </is>
-      </c>
-      <c r="B18" s="6">
-        <f>B16+B17</f>
-        <v/>
-      </c>
-      <c r="C18" s="2" t="inlineStr">
-        <is>
-          <t>PHP/month</t>
-        </is>
-      </c>
-      <c r="D18" s="2" t="inlineStr">
-        <is>
-          <t>Total revenue</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr">
-        <is>
-          <t>Rider base payroll</t>
-        </is>
-      </c>
-      <c r="B19" s="6">
-        <f>Inputs!B9*Inputs!B26*Inputs!B12*(1+Inputs!B27)</f>
-        <v/>
-      </c>
-      <c r="C19" s="2" t="inlineStr">
-        <is>
-          <t>PHP/month</t>
-        </is>
-      </c>
-      <c r="D19" s="2" t="inlineStr">
-        <is>
-          <t>Wages plus burden</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>Gross fare / rider / day</t>
-        </is>
-      </c>
-      <c r="B20" s="6">
-        <f>(B13*B9)/(Inputs!B9*Inputs!B12)</f>
-        <v/>
-      </c>
-      <c r="C20" s="2" t="inlineStr">
-        <is>
-          <t>PHP/rider/day</t>
-        </is>
-      </c>
-      <c r="D20" s="2" t="inlineStr">
-        <is>
-          <t>Incentive basis</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="2" t="inlineStr">
-        <is>
-          <t>Rider incentives</t>
-        </is>
-      </c>
-      <c r="B21" s="6">
-        <f>Inputs!B9*Inputs!B12*MAX(B20-Inputs!B28,0)*Inputs!B29</f>
-        <v/>
-      </c>
-      <c r="C21" s="2" t="inlineStr">
-        <is>
-          <t>PHP/month</t>
-        </is>
-      </c>
-      <c r="D21" s="2" t="inlineStr">
-        <is>
-          <t>Commission above threshold</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="2" t="inlineStr">
-        <is>
-          <t>Electricity</t>
-        </is>
-      </c>
-      <c r="B22" s="6">
-        <f>B13*Inputs!B14*Inputs!B35*Inputs!B36</f>
-        <v/>
-      </c>
-      <c r="C22" s="2" t="inlineStr">
-        <is>
-          <t>PHP/month</t>
-        </is>
-      </c>
-      <c r="D22" s="2" t="inlineStr">
-        <is>
-          <t>Charging cost</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="2" t="inlineStr">
-        <is>
-          <t>Fleet acquisition / amortization</t>
-        </is>
-      </c>
-      <c r="B23" s="6">
-        <f>IF(Inputs!B5=1,Inputs!B9*(Inputs!B30+Inputs!B31)/Inputs!B32,0)</f>
-        <v/>
-      </c>
-      <c r="C23" s="2" t="inlineStr">
-        <is>
-          <t>PHP/month</t>
-        </is>
-      </c>
-      <c r="D23" s="2" t="inlineStr">
-        <is>
-          <t>Asset recovery switch</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="2" t="inlineStr">
-        <is>
-          <t>Fleet maintenance, insurance, registration</t>
-        </is>
-      </c>
-      <c r="B24" s="6">
-        <f>Inputs!B9*(Inputs!B33+Inputs!B34)</f>
-        <v/>
-      </c>
-      <c r="C24" s="2" t="inlineStr">
-        <is>
-          <t>PHP/month</t>
-        </is>
-      </c>
-      <c r="D24" s="2" t="inlineStr">
-        <is>
-          <t>Fleet operating cost</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="2" t="inlineStr">
-        <is>
-          <t>Development build recovery</t>
-        </is>
-      </c>
-      <c r="B25" s="6">
-        <f>IF(Inputs!B6=1,Inputs!B37/Inputs!B38,0)</f>
-        <v/>
-      </c>
-      <c r="C25" s="2" t="inlineStr">
-        <is>
-          <t>PHP/month</t>
-        </is>
-      </c>
-      <c r="D25" s="2" t="inlineStr">
-        <is>
-          <t>Build recovery switch</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="2" t="inlineStr">
-        <is>
-          <t>Ongoing dev support retainer</t>
-        </is>
-      </c>
-      <c r="B26" s="6">
-        <f>IF(Inputs!B6=1,Inputs!B39,0)</f>
-        <v/>
-      </c>
-      <c r="C26" s="2" t="inlineStr">
-        <is>
-          <t>PHP/month</t>
-        </is>
-      </c>
-      <c r="D26" s="2" t="inlineStr">
-        <is>
-          <t>Dev support switch</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="2" t="inlineStr">
-        <is>
-          <t>Cloud / API cost</t>
-        </is>
-      </c>
-      <c r="B27" s="6">
-        <f>IF(Inputs!B7=1,Cloud_Tiers!B8,0)</f>
-        <v/>
-      </c>
-      <c r="C27" s="2" t="inlineStr">
-        <is>
-          <t>PHP/month</t>
-        </is>
-      </c>
-      <c r="D27" s="2" t="inlineStr">
-        <is>
-          <t>Cloud recovery switch</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="2" t="inlineStr">
-        <is>
-          <t>Operations, support and admin</t>
-        </is>
-      </c>
-      <c r="B28" s="6">
-        <f>Inputs!B41+Inputs!B8*(Inputs!B42+Inputs!B43)</f>
-        <v/>
-      </c>
-      <c r="C28" s="2" t="inlineStr">
-        <is>
-          <t>PHP/month</t>
-        </is>
-      </c>
-      <c r="D28" s="2" t="inlineStr">
-        <is>
-          <t>Fixed + user ops</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="2" t="inlineStr">
-        <is>
-          <t>Payment processing</t>
-        </is>
-      </c>
-      <c r="B29" s="6">
-        <f>B18*Inputs!B44*Inputs!B45</f>
-        <v/>
-      </c>
-      <c r="C29" s="2" t="inlineStr">
-        <is>
-          <t>PHP/month</t>
-        </is>
-      </c>
-      <c r="D29" s="2" t="inlineStr">
-        <is>
-          <t>Digital payment fee</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="2" t="inlineStr">
-        <is>
-          <t>Tax / regulatory reserve</t>
-        </is>
-      </c>
-      <c r="B30" s="6">
-        <f>B18*Inputs!B46</f>
-        <v/>
-      </c>
-      <c r="C30" s="2" t="inlineStr">
-        <is>
-          <t>PHP/month</t>
-        </is>
-      </c>
-      <c r="D30" s="2" t="inlineStr">
-        <is>
-          <t>Revenue reserve</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="2" t="inlineStr">
-        <is>
-          <t>Total cost</t>
-        </is>
-      </c>
-      <c r="B31" s="6">
-        <f>SUM(B19,B21:B29)</f>
-        <v/>
-      </c>
-      <c r="C31" s="2" t="inlineStr">
-        <is>
-          <t>PHP/month</t>
-        </is>
-      </c>
-      <c r="D31" s="2" t="inlineStr">
-        <is>
-          <t>Total monthly cost</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="2" t="inlineStr">
-        <is>
-          <t>Monthly profit / loss</t>
-        </is>
-      </c>
-      <c r="B32" s="6">
-        <f>B18-B31</f>
-        <v/>
-      </c>
-      <c r="C32" s="2" t="inlineStr">
-        <is>
-          <t>PHP/month</t>
-        </is>
-      </c>
-      <c r="D32" s="2" t="inlineStr">
-        <is>
-          <t>Net result</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="2" t="inlineStr">
-        <is>
-          <t>Required revenue / active user</t>
-        </is>
-      </c>
-      <c r="B33" s="6">
-        <f>B31/Inputs!B8</f>
-        <v/>
-      </c>
-      <c r="C33" s="2" t="inlineStr">
-        <is>
-          <t>PHP/user/month</t>
-        </is>
-      </c>
-      <c r="D33" s="2" t="inlineStr">
-        <is>
-          <t>Cost to recover per active user</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="2" t="inlineStr">
-        <is>
-          <t>Revenue / active user</t>
-        </is>
-      </c>
-      <c r="B34" s="6">
-        <f>B18/Inputs!B8</f>
-        <v/>
-      </c>
-      <c r="C34" s="2" t="inlineStr">
-        <is>
-          <t>PHP/user/month</t>
-        </is>
-      </c>
-      <c r="D34" s="2" t="inlineStr">
-        <is>
-          <t>Current revenue per active user</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="2" t="inlineStr">
-        <is>
-          <t>Profit / active user</t>
-        </is>
-      </c>
-      <c r="B35" s="6">
-        <f>B32/Inputs!B8</f>
-        <v/>
-      </c>
-      <c r="C35" s="2" t="inlineStr">
-        <is>
-          <t>PHP/user/month</t>
-        </is>
-      </c>
-      <c r="D35" s="2" t="inlineStr">
-        <is>
-          <t>Net per active user</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="2" t="inlineStr">
-        <is>
-          <t>Cost / completed ride</t>
-        </is>
-      </c>
-      <c r="B36" s="6">
-        <f>B31/B13</f>
-        <v/>
-      </c>
-      <c r="C36" s="2" t="inlineStr">
-        <is>
-          <t>PHP/ride</t>
-        </is>
-      </c>
-      <c r="D36" s="2" t="inlineStr">
-        <is>
-          <t>Average cost per ride</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="2" t="inlineStr">
-        <is>
-          <t>Profit / completed ride</t>
-        </is>
-      </c>
-      <c r="B37" s="7">
-        <f>B32/B13</f>
-        <v/>
-      </c>
-      <c r="C37" s="2" t="inlineStr">
-        <is>
-          <t>PHP/ride</t>
-        </is>
-      </c>
-      <c r="D37" s="2" t="inlineStr">
-        <is>
-          <t>Average profit per ride</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="2" t="inlineStr">
-        <is>
-          <t>Fleet utilization</t>
-        </is>
-      </c>
-      <c r="B38" s="6">
-        <f>B12/B11</f>
-        <v/>
-      </c>
-      <c r="C38" s="2" t="inlineStr">
-        <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="D38" s="2" t="inlineStr">
-        <is>
-          <t>Served requested rides / capacity</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="2" t="inlineStr">
-        <is>
-          <t>Approx. break-even completed rides/month</t>
-        </is>
-      </c>
-      <c r="B39" s="6">
-        <f>IF((B9*Inputs!B24*(1-Inputs!B44*Inputs!B45-Inputs!B46)-Inputs!B14*Inputs!B35*Inputs!B36)&gt;0,(B19+B21+B23+B24+B25+B26+B27+B28)/(B9*Inputs!B24*(1-Inputs!B44*Inputs!B45-Inputs!B46)-Inputs!B14*Inputs!B35*Inputs!B36),"Check fare")</f>
-        <v/>
-      </c>
-      <c r="C39" s="2" t="inlineStr">
-        <is>
-          <t>rides/month</t>
-        </is>
-      </c>
-      <c r="D39" s="2" t="inlineStr">
-        <is>
-          <t>Approximate target; keeps incentive at current threshold behavior</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="2" t="inlineStr">
-        <is>
-          <t>Approx. break-even completed rides/day</t>
-        </is>
-      </c>
-      <c r="B40" s="6">
-        <f>B39/Inputs!B12</f>
-        <v/>
-      </c>
-      <c r="C40" s="2" t="inlineStr">
-        <is>
-          <t>rides/day</t>
-        </is>
-      </c>
-      <c r="D40" s="2" t="inlineStr">
-        <is>
-          <t>Daily target</t>
-        </is>
+      <c r="A6" s="13" t="inlineStr">
+        <is>
+          <t>Profitable utilization case</t>
+        </is>
+      </c>
+      <c r="B6" s="16" t="n">
+        <v>6000</v>
+      </c>
+      <c r="C6" s="16" t="n">
+        <v>50</v>
+      </c>
+      <c r="D6" s="17" t="n">
+        <v>8</v>
+      </c>
+      <c r="E6" s="17" t="n">
+        <v>20</v>
+      </c>
+      <c r="F6" s="17">
+        <f>MIN(B6*D6,C6*E6*Inputs!B12)*Inputs!B13/(C6*Inputs!B12)</f>
+        <v/>
+      </c>
+      <c r="G6" s="17">
+        <f>MIN(B6*D6,C6*E6*Inputs!B12)*Inputs!B13*Model!B9/(C6*Inputs!B12)</f>
+        <v/>
+      </c>
+      <c r="H6" s="17">
+        <f>Inputs!B26*(1+Inputs!B27)</f>
+        <v/>
+      </c>
+      <c r="I6" s="18">
+        <f>G6/H6</f>
+        <v/>
+      </c>
+      <c r="J6" s="17">
+        <f>((MIN(B6*D6,C6*E6*Inputs!B12)*Inputs!B13)*Model!B9*Inputs!B24 + B6*Inputs!B25) - (C6*Inputs!B26*Inputs!B12*(1+Inputs!B27) + C6*Inputs!B12*MAX(G6-Inputs!B28,0)*Inputs!B29 + (MIN(B6*D6,C6*E6*Inputs!B12)*Inputs!B13)*Inputs!B14*Inputs!B35*Inputs!B36 + IF(Inputs!B5=1,C6*(Inputs!B30+Inputs!B31)/Inputs!B32,0) + C6*(Inputs!B33+Inputs!B34) + IF(Inputs!B6=1,Inputs!B37/Inputs!B38+Inputs!B39,0) + IF(Inputs!B7=1,Inputs!B40+SUM(MAX(B6*21*5-10000,0)/1000*2.83,MAX(B6*21*2-10000,0)/1000*5,MAX(B6*21*1-10000,0)/1000*5,MAX(B6*21*2-10000,0)/1000*5)*58,0) + Inputs!B41+B6*(Inputs!B42+Inputs!B43) + ((MIN(B6*D6,C6*E6*Inputs!B12)*Inputs!B13)*Model!B9*Inputs!B24+B6*Inputs!B25)*Inputs!B44*Inputs!B45 + ((MIN(B6*D6,C6*E6*Inputs!B12)*Inputs!B13)*Model!B9*Inputs!B24+B6*Inputs!B25)*Inputs!B46)</f>
+        <v/>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -2458,19 +2240,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D15"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:D40"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
-    <col width="42" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="48" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="23.4" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Monthly Cost Breakdown</t>
+          <t>E-Ride Operating Model - Calculations</t>
         </is>
       </c>
       <c r="B1" s="2" t="n"/>
@@ -2480,7 +2262,7 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Cost lines link directly to Model calculations.</t>
+          <t>Core deterministic calculation. This is the Excel fallback for the dashboard.</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -2496,237 +2278,783 @@
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>Cost category</t>
+          <t>Metric</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>Monthly PHP</t>
+          <t>Formula / Value</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>Share of cost</t>
+          <t>Unit</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>PHP / completed ride</t>
+          <t>Meaning</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Rider base payroll</t>
+          <t>Short distance km</t>
         </is>
       </c>
       <c r="B5" s="6">
-        <f>Model!B19</f>
-        <v/>
-      </c>
-      <c r="C5" s="7">
-        <f>B5/Model!B31</f>
-        <v/>
-      </c>
-      <c r="D5" s="6">
-        <f>B5/Model!B13</f>
-        <v/>
+        <f>MIN(MAX(Inputs!B14-Inputs!B17,0),MAX(Inputs!B19-Inputs!B17,0))</f>
+        <v/>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>km</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Charged at regular per-km rate</t>
+        </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Rider incentives</t>
+          <t>Long distance km</t>
         </is>
       </c>
       <c r="B6" s="6">
-        <f>Model!B21</f>
-        <v/>
-      </c>
-      <c r="C6" s="7">
-        <f>B6/Model!B31</f>
-        <v/>
-      </c>
-      <c r="D6" s="6">
-        <f>B6/Model!B13</f>
-        <v/>
+        <f>MAX(Inputs!B14-Inputs!B19,0)</f>
+        <v/>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>km</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Charged at long-distance rate</t>
+        </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Electricity</t>
+          <t>Charged minutes</t>
         </is>
       </c>
       <c r="B7" s="6">
-        <f>Model!B22</f>
-        <v/>
-      </c>
-      <c r="C7" s="7">
-        <f>B7/Model!B31</f>
-        <v/>
-      </c>
-      <c r="D7" s="6">
-        <f>B7/Model!B13</f>
-        <v/>
+        <f>MAX(Inputs!B15-Inputs!B21,0)</f>
+        <v/>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>minutes</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Charged beyond base minutes</t>
+        </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Fleet acquisition / amortization</t>
+          <t>Fare before discount</t>
         </is>
       </c>
       <c r="B8" s="6">
-        <f>Model!B23</f>
-        <v/>
-      </c>
-      <c r="C8" s="7">
-        <f>B8/Model!B31</f>
-        <v/>
-      </c>
-      <c r="D8" s="6">
-        <f>B8/Model!B13</f>
-        <v/>
+        <f>Inputs!B16+B5*Inputs!B18+B6*Inputs!B20+B7*Inputs!B22</f>
+        <v/>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>PHP/ride</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Benchmark fare</t>
+        </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Fleet maintenance, insurance, registration</t>
+          <t>Final passenger fare</t>
         </is>
       </c>
       <c r="B9" s="6">
-        <f>Model!B24</f>
-        <v/>
-      </c>
-      <c r="C9" s="7">
-        <f>B9/Model!B31</f>
-        <v/>
-      </c>
-      <c r="D9" s="6">
-        <f>B9/Model!B13</f>
-        <v/>
+        <f>B8*(1-Inputs!B23)</f>
+        <v/>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>PHP/ride</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Passenger fare</t>
+        </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Development build recovery</t>
+          <t>Requested demand</t>
         </is>
       </c>
       <c r="B10" s="6">
-        <f>Model!B25</f>
-        <v/>
-      </c>
-      <c r="C10" s="7">
-        <f>B10/Model!B31</f>
-        <v/>
-      </c>
-      <c r="D10" s="6">
-        <f>B10/Model!B13</f>
-        <v/>
+        <f>Inputs!B8*Inputs!B10</f>
+        <v/>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>rides/month</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>User demand</t>
+        </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Ongoing dev support retainer</t>
+          <t>Requested fleet capacity</t>
         </is>
       </c>
       <c r="B11" s="6">
-        <f>Model!B26</f>
-        <v/>
-      </c>
-      <c r="C11" s="7">
-        <f>B11/Model!B31</f>
-        <v/>
-      </c>
-      <c r="D11" s="6">
-        <f>B11/Model!B13</f>
-        <v/>
+        <f>Inputs!B9*Inputs!B11*Inputs!B12</f>
+        <v/>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>rides/month</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Fleet capacity</t>
+        </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Cloud / API cost</t>
+          <t>Requested served rides</t>
         </is>
       </c>
       <c r="B12" s="6">
-        <f>Model!B27</f>
-        <v/>
-      </c>
-      <c r="C12" s="7">
-        <f>B12/Model!B31</f>
-        <v/>
-      </c>
-      <c r="D12" s="6">
-        <f>B12/Model!B13</f>
-        <v/>
+        <f>MIN(B10,B11)</f>
+        <v/>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>rides/month</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Matched rides</t>
+        </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Operations, support and admin</t>
+          <t>Completed rides</t>
         </is>
       </c>
       <c r="B13" s="6">
-        <f>Model!B28</f>
-        <v/>
-      </c>
-      <c r="C13" s="7">
-        <f>B13/Model!B31</f>
-        <v/>
-      </c>
-      <c r="D13" s="6">
-        <f>B13/Model!B13</f>
-        <v/>
+        <f>B12*Inputs!B13</f>
+        <v/>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>rides/month</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>Revenue-generating rides</t>
+        </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Payment processing</t>
+          <t>Completed rides / day</t>
         </is>
       </c>
       <c r="B14" s="6">
-        <f>Model!B29</f>
-        <v/>
-      </c>
-      <c r="C14" s="7">
-        <f>B14/Model!B31</f>
-        <v/>
-      </c>
-      <c r="D14" s="6">
-        <f>B14/Model!B13</f>
-        <v/>
+        <f>B13/Inputs!B12</f>
+        <v/>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>rides/day</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Daily completed rides</t>
+        </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
+          <t>Completed rides / rider / day</t>
+        </is>
+      </c>
+      <c r="B15" s="6">
+        <f>B13/(Inputs!B9*Inputs!B12)</f>
+        <v/>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>rides/rider/day</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>Actual utilization</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Fare revenue</t>
+        </is>
+      </c>
+      <c r="B16" s="6">
+        <f>B13*B9*Inputs!B24</f>
+        <v/>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>PHP/month</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>Retained fare revenue</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>Membership revenue</t>
+        </is>
+      </c>
+      <c r="B17" s="6">
+        <f>Inputs!B8*Inputs!B25</f>
+        <v/>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>PHP/month</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>Optional user fees</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>Total revenue</t>
+        </is>
+      </c>
+      <c r="B18" s="6">
+        <f>B16+B17</f>
+        <v/>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>PHP/month</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>Total revenue</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>Rider base payroll</t>
+        </is>
+      </c>
+      <c r="B19" s="6">
+        <f>Inputs!B9*Inputs!B26*Inputs!B12*(1+Inputs!B27)</f>
+        <v/>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>PHP/month</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>Wages plus burden</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>Gross fare / rider / day</t>
+        </is>
+      </c>
+      <c r="B20" s="6">
+        <f>(B13*B9)/(Inputs!B9*Inputs!B12)</f>
+        <v/>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>PHP/rider/day</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>Incentive basis</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>Rider incentives</t>
+        </is>
+      </c>
+      <c r="B21" s="6">
+        <f>Inputs!B9*Inputs!B12*MAX(B20-Inputs!B28,0)*Inputs!B29</f>
+        <v/>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>PHP/month</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>Commission above threshold</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>Electricity</t>
+        </is>
+      </c>
+      <c r="B22" s="6">
+        <f>B13*Inputs!B14*Inputs!B35*Inputs!B36</f>
+        <v/>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>PHP/month</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>Charging cost</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>Fleet acquisition / amortization</t>
+        </is>
+      </c>
+      <c r="B23" s="6">
+        <f>IF(Inputs!B5=1,Inputs!B9*(Inputs!B30+Inputs!B31)/Inputs!B32,0)</f>
+        <v/>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>PHP/month</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>Asset recovery switch</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>Fleet maintenance, insurance, registration</t>
+        </is>
+      </c>
+      <c r="B24" s="6">
+        <f>Inputs!B9*(Inputs!B33+Inputs!B34)</f>
+        <v/>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>PHP/month</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>Fleet operating cost</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>Development build recovery</t>
+        </is>
+      </c>
+      <c r="B25" s="6">
+        <f>IF(Inputs!B6=1,Inputs!B37/Inputs!B38,0)</f>
+        <v/>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>PHP/month</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>Build recovery switch</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>Ongoing dev support retainer</t>
+        </is>
+      </c>
+      <c r="B26" s="6">
+        <f>IF(Inputs!B6=1,Inputs!B39,0)</f>
+        <v/>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>PHP/month</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>Dev support switch</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>Cloud / API cost</t>
+        </is>
+      </c>
+      <c r="B27" s="6">
+        <f>IF(Inputs!B7=1,Cloud_Tiers!B8,0)</f>
+        <v/>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>PHP/month</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>Cloud recovery switch</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>Operations, support and admin</t>
+        </is>
+      </c>
+      <c r="B28" s="6">
+        <f>Inputs!B41+Inputs!B8*(Inputs!B42+Inputs!B43)</f>
+        <v/>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>PHP/month</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>Fixed + user ops</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>Payment processing</t>
+        </is>
+      </c>
+      <c r="B29" s="6">
+        <f>B18*Inputs!B44*Inputs!B45</f>
+        <v/>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>PHP/month</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>Digital payment fee</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
           <t>Tax / regulatory reserve</t>
         </is>
       </c>
-      <c r="B15" s="6">
-        <f>Model!B30</f>
-        <v/>
-      </c>
-      <c r="C15" s="7">
-        <f>B15/Model!B31</f>
-        <v/>
-      </c>
-      <c r="D15" s="6">
-        <f>B15/Model!B13</f>
-        <v/>
+      <c r="B30" s="6">
+        <f>B18*Inputs!B46</f>
+        <v/>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>PHP/month</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>Revenue reserve</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>Total cost</t>
+        </is>
+      </c>
+      <c r="B31" s="6">
+        <f>SUM(B19,B21:B29)</f>
+        <v/>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>PHP/month</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>Total monthly cost</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>Monthly profit / loss</t>
+        </is>
+      </c>
+      <c r="B32" s="6">
+        <f>B18-B31</f>
+        <v/>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>PHP/month</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>Net result</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>Required revenue / active user</t>
+        </is>
+      </c>
+      <c r="B33" s="6">
+        <f>B31/Inputs!B8</f>
+        <v/>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>PHP/user/month</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>Cost to recover per active user</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>Revenue / active user</t>
+        </is>
+      </c>
+      <c r="B34" s="6">
+        <f>B18/Inputs!B8</f>
+        <v/>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>PHP/user/month</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>Current revenue per active user</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>Profit / active user</t>
+        </is>
+      </c>
+      <c r="B35" s="6">
+        <f>B32/Inputs!B8</f>
+        <v/>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>PHP/user/month</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>Net per active user</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>Cost / completed ride</t>
+        </is>
+      </c>
+      <c r="B36" s="6">
+        <f>B31/B13</f>
+        <v/>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>PHP/ride</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>Average cost per ride</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>Profit / completed ride</t>
+        </is>
+      </c>
+      <c r="B37" s="7">
+        <f>B32/B13</f>
+        <v/>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>PHP/ride</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>Average profit per ride</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>Fleet utilization</t>
+        </is>
+      </c>
+      <c r="B38" s="6">
+        <f>B12/B11</f>
+        <v/>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>Served requested rides / capacity</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>Approx. break-even completed rides/month</t>
+        </is>
+      </c>
+      <c r="B39" s="6">
+        <f>IF((B9*Inputs!B24*(1-Inputs!B44*Inputs!B45-Inputs!B46)-Inputs!B14*Inputs!B35*Inputs!B36)&gt;0,(B19+B21+B23+B24+B25+B26+B27+B28)/(B9*Inputs!B24*(1-Inputs!B44*Inputs!B45-Inputs!B46)-Inputs!B14*Inputs!B35*Inputs!B36),"Check fare")</f>
+        <v/>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>rides/month</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>Approximate target; keeps incentive at current threshold behavior</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>Approx. break-even completed rides/day</t>
+        </is>
+      </c>
+      <c r="B40" s="6">
+        <f>B39/Inputs!B12</f>
+        <v/>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>rides/day</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>Daily target</t>
+        </is>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -2736,19 +3064,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D12"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:D15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="42" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="23.4" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>AWS / Cloud and API Cost Tiers</t>
+          <t>Monthly Cost Breakdown</t>
         </is>
       </c>
       <c r="B1" s="2" t="n"/>
@@ -2758,7 +3085,7 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Uses the workbook-based Google Maps/API scaling plus POC baseline.</t>
+          <t>Cost lines link directly to Model calculations.</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -2774,167 +3101,231 @@
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>Tier</t>
+          <t>Cost category</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>Estimated monthly cloud/API cost</t>
+          <t>Monthly PHP</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>Active users</t>
+          <t>Share of cost</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>Cost / active user</t>
+          <t>PHP / completed ride</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>POC pilot</t>
+          <t>Rider base payroll</t>
         </is>
       </c>
       <c r="B5" s="6">
-        <f>Inputs!B40+SUM(MAX(C5*21*5-10000,0)/1000*2.83,MAX(C5*21*2-10000,0)/1000*5,MAX(C5*21*1-10000,0)/1000*5,MAX(C5*21*2-10000,0)/1000*5)*58</f>
-        <v/>
-      </c>
-      <c r="C5" s="8" t="n">
-        <v>20</v>
+        <f>Model!B19</f>
+        <v/>
+      </c>
+      <c r="C5" s="7">
+        <f>B5/Model!B31</f>
+        <v/>
       </c>
       <c r="D5" s="6">
-        <f>B5/C5</f>
+        <f>B5/Model!B13</f>
         <v/>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Small internal launch</t>
+          <t>Rider incentives</t>
         </is>
       </c>
       <c r="B6" s="6">
-        <f>Inputs!B40+SUM(MAX(C6*21*5-10000,0)/1000*2.83,MAX(C6*21*2-10000,0)/1000*5,MAX(C6*21*1-10000,0)/1000*5,MAX(C6*21*2-10000,0)/1000*5)*58</f>
-        <v/>
-      </c>
-      <c r="C6" s="8" t="n">
-        <v>100</v>
+        <f>Model!B21</f>
+        <v/>
+      </c>
+      <c r="C6" s="7">
+        <f>B6/Model!B31</f>
+        <v/>
       </c>
       <c r="D6" s="6">
-        <f>B6/C6</f>
+        <f>B6/Model!B13</f>
         <v/>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Campus/barangay launch</t>
+          <t>Electricity</t>
         </is>
       </c>
       <c r="B7" s="6">
-        <f>Inputs!B40+SUM(MAX(C7*21*5-10000,0)/1000*2.83,MAX(C7*21*2-10000,0)/1000*5,MAX(C7*21*1-10000,0)/1000*5,MAX(C7*21*2-10000,0)/1000*5)*58</f>
-        <v/>
-      </c>
-      <c r="C7" s="8" t="n">
-        <v>500</v>
+        <f>Model!B22</f>
+        <v/>
+      </c>
+      <c r="C7" s="7">
+        <f>B7/Model!B31</f>
+        <v/>
       </c>
       <c r="D7" s="6">
-        <f>B7/C7</f>
+        <f>B7/Model!B13</f>
         <v/>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Early city launch</t>
+          <t>Fleet acquisition / amortization</t>
         </is>
       </c>
       <c r="B8" s="6">
-        <f>Inputs!B40+SUM(MAX(C8*21*5-10000,0)/1000*2.83,MAX(C8*21*2-10000,0)/1000*5,MAX(C8*21*1-10000,0)/1000*5,MAX(C8*21*2-10000,0)/1000*5)*58</f>
-        <v/>
-      </c>
-      <c r="C8" s="8" t="n">
-        <v>1000</v>
+        <f>Model!B23</f>
+        <v/>
+      </c>
+      <c r="C8" s="7">
+        <f>B8/Model!B31</f>
+        <v/>
       </c>
       <c r="D8" s="6">
-        <f>B8/C8</f>
+        <f>B8/Model!B13</f>
         <v/>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Current scenario</t>
+          <t>Fleet maintenance, insurance, registration</t>
         </is>
       </c>
       <c r="B9" s="6">
-        <f>Inputs!B40+SUM(MAX(C9*21*5-10000,0)/1000*2.83,MAX(C9*21*2-10000,0)/1000*5,MAX(C9*21*1-10000,0)/1000*5,MAX(C9*21*2-10000,0)/1000*5)*58</f>
-        <v/>
-      </c>
-      <c r="C9" s="8">
-        <f>Inputs!B8</f>
+        <f>Model!B24</f>
+        <v/>
+      </c>
+      <c r="C9" s="7">
+        <f>B9/Model!B31</f>
         <v/>
       </c>
       <c r="D9" s="6">
-        <f>B9/C9</f>
+        <f>B9/Model!B13</f>
         <v/>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Dense launch</t>
+          <t>Development build recovery</t>
         </is>
       </c>
       <c r="B10" s="6">
-        <f>Inputs!B40+SUM(MAX(C10*21*5-10000,0)/1000*2.83,MAX(C10*21*2-10000,0)/1000*5,MAX(C10*21*1-10000,0)/1000*5,MAX(C10*21*2-10000,0)/1000*5)*58</f>
-        <v/>
-      </c>
-      <c r="C10" s="8" t="n">
-        <v>5000</v>
+        <f>Model!B25</f>
+        <v/>
+      </c>
+      <c r="C10" s="7">
+        <f>B10/Model!B31</f>
+        <v/>
       </c>
       <c r="D10" s="6">
-        <f>B10/C10</f>
+        <f>B10/Model!B13</f>
         <v/>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>City scale</t>
+          <t>Ongoing dev support retainer</t>
         </is>
       </c>
       <c r="B11" s="6">
-        <f>Inputs!B40+SUM(MAX(C11*21*5-10000,0)/1000*2.83,MAX(C11*21*2-10000,0)/1000*5,MAX(C11*21*1-10000,0)/1000*5,MAX(C11*21*2-10000,0)/1000*5)*58</f>
-        <v/>
-      </c>
-      <c r="C11" s="8" t="n">
-        <v>10000</v>
+        <f>Model!B26</f>
+        <v/>
+      </c>
+      <c r="C11" s="7">
+        <f>B11/Model!B31</f>
+        <v/>
       </c>
       <c r="D11" s="6">
-        <f>B11/C11</f>
+        <f>B11/Model!B13</f>
         <v/>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Metro scale stress test</t>
+          <t>Cloud / API cost</t>
         </is>
       </c>
       <c r="B12" s="6">
-        <f>Inputs!B40+SUM(MAX(C12*21*5-10000,0)/1000*2.83,MAX(C12*21*2-10000,0)/1000*5,MAX(C12*21*1-10000,0)/1000*5,MAX(C12*21*2-10000,0)/1000*5)*58</f>
-        <v/>
-      </c>
-      <c r="C12" s="8" t="n">
-        <v>25000</v>
+        <f>Model!B27</f>
+        <v/>
+      </c>
+      <c r="C12" s="7">
+        <f>B12/Model!B31</f>
+        <v/>
       </c>
       <c r="D12" s="6">
-        <f>B12/C12</f>
+        <f>B12/Model!B13</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Operations, support and admin</t>
+        </is>
+      </c>
+      <c r="B13" s="6">
+        <f>Model!B28</f>
+        <v/>
+      </c>
+      <c r="C13" s="7">
+        <f>B13/Model!B31</f>
+        <v/>
+      </c>
+      <c r="D13" s="6">
+        <f>B13/Model!B13</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Payment processing</t>
+        </is>
+      </c>
+      <c r="B14" s="6">
+        <f>Model!B29</f>
+        <v/>
+      </c>
+      <c r="C14" s="7">
+        <f>B14/Model!B31</f>
+        <v/>
+      </c>
+      <c r="D14" s="6">
+        <f>B14/Model!B13</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Tax / regulatory reserve</t>
+        </is>
+      </c>
+      <c r="B15" s="6">
+        <f>Model!B30</f>
+        <v/>
+      </c>
+      <c r="C15" s="7">
+        <f>B15/Model!B31</f>
+        <v/>
+      </c>
+      <c r="D15" s="6">
+        <f>B15/Model!B13</f>
         <v/>
       </c>
     </row>
@@ -2951,18 +3342,18 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:D12"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
-    <col width="38" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="23.4" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Development Budget Allocation</t>
+          <t>AWS / Cloud and API Cost Tiers</t>
         </is>
       </c>
       <c r="B1" s="2" t="n"/>
@@ -2972,7 +3363,7 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Default allocation sums to PHP 1,000,000 and scales with the editable build budget.</t>
+          <t>Uses the workbook-based Google Maps/API scaling plus POC baseline.</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -2988,179 +3379,173 @@
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>Role</t>
+          <t>Tier</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>6-month allocation</t>
+          <t>Estimated monthly cloud/API cost</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>Monthly allocation</t>
+          <t>Active users</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>Share</t>
+          <t>Cost / active user</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Lead full-stack developer / PM</t>
+          <t>POC pilot</t>
         </is>
       </c>
       <c r="B5" s="6">
-        <f>330000/1000000*Inputs!B37</f>
-        <v/>
-      </c>
-      <c r="C5" s="6">
-        <f>B5/6</f>
-        <v/>
-      </c>
-      <c r="D5" s="7">
-        <f>B5/SUM($B$5:$B$11)</f>
+        <f>Inputs!B40+SUM(MAX(C5*21*5-10000,0)/1000*2.83,MAX(C5*21*2-10000,0)/1000*5,MAX(C5*21*1-10000,0)/1000*5,MAX(C5*21*2-10000,0)/1000*5)*58</f>
+        <v/>
+      </c>
+      <c r="C5" s="8" t="n">
+        <v>20</v>
+      </c>
+      <c r="D5" s="6">
+        <f>B5/C5</f>
         <v/>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Backend developer</t>
+          <t>Small internal launch</t>
         </is>
       </c>
       <c r="B6" s="6">
-        <f>180000/1000000*Inputs!B37</f>
-        <v/>
-      </c>
-      <c r="C6" s="6">
-        <f>B6/6</f>
-        <v/>
-      </c>
-      <c r="D6" s="7">
-        <f>B6/SUM($B$5:$B$11)</f>
+        <f>Inputs!B40+SUM(MAX(C6*21*5-10000,0)/1000*2.83,MAX(C6*21*2-10000,0)/1000*5,MAX(C6*21*1-10000,0)/1000*5,MAX(C6*21*2-10000,0)/1000*5)*58</f>
+        <v/>
+      </c>
+      <c r="C6" s="8" t="n">
+        <v>100</v>
+      </c>
+      <c r="D6" s="6">
+        <f>B6/C6</f>
         <v/>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Frontend/mobile developer</t>
+          <t>Campus/barangay launch</t>
         </is>
       </c>
       <c r="B7" s="6">
-        <f>140000/1000000*Inputs!B37</f>
-        <v/>
-      </c>
-      <c r="C7" s="6">
-        <f>B7/6</f>
-        <v/>
-      </c>
-      <c r="D7" s="7">
-        <f>B7/SUM($B$5:$B$11)</f>
+        <f>Inputs!B40+SUM(MAX(C7*21*5-10000,0)/1000*2.83,MAX(C7*21*2-10000,0)/1000*5,MAX(C7*21*1-10000,0)/1000*5,MAX(C7*21*2-10000,0)/1000*5)*58</f>
+        <v/>
+      </c>
+      <c r="C7" s="8" t="n">
+        <v>500</v>
+      </c>
+      <c r="D7" s="6">
+        <f>B7/C7</f>
         <v/>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Cloud / DevOps engineer</t>
+          <t>Early city launch</t>
         </is>
       </c>
       <c r="B8" s="6">
-        <f>120000/1000000*Inputs!B37</f>
-        <v/>
-      </c>
-      <c r="C8" s="6">
-        <f>B8/6</f>
-        <v/>
-      </c>
-      <c r="D8" s="7">
-        <f>B8/SUM($B$5:$B$11)</f>
+        <f>Inputs!B40+SUM(MAX(C8*21*5-10000,0)/1000*2.83,MAX(C8*21*2-10000,0)/1000*5,MAX(C8*21*1-10000,0)/1000*5,MAX(C8*21*2-10000,0)/1000*5)*58</f>
+        <v/>
+      </c>
+      <c r="C8" s="8" t="n">
+        <v>1000</v>
+      </c>
+      <c r="D8" s="6">
+        <f>B8/C8</f>
         <v/>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>QA and release support</t>
+          <t>Current scenario</t>
         </is>
       </c>
       <c r="B9" s="6">
-        <f>90000/1000000*Inputs!B37</f>
-        <v/>
-      </c>
-      <c r="C9" s="6">
-        <f>B9/6</f>
-        <v/>
-      </c>
-      <c r="D9" s="7">
-        <f>B9/SUM($B$5:$B$11)</f>
+        <f>Inputs!B40+SUM(MAX(C9*21*5-10000,0)/1000*2.83,MAX(C9*21*2-10000,0)/1000*5,MAX(C9*21*1-10000,0)/1000*5,MAX(C9*21*2-10000,0)/1000*5)*58</f>
+        <v/>
+      </c>
+      <c r="C9" s="8">
+        <f>Inputs!B8</f>
+        <v/>
+      </c>
+      <c r="D9" s="6">
+        <f>B9/C9</f>
         <v/>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Product / client coordination</t>
+          <t>Dense launch</t>
         </is>
       </c>
       <c r="B10" s="6">
-        <f>80000/1000000*Inputs!B37</f>
-        <v/>
-      </c>
-      <c r="C10" s="6">
-        <f>B10/6</f>
-        <v/>
-      </c>
-      <c r="D10" s="7">
-        <f>B10/SUM($B$5:$B$11)</f>
+        <f>Inputs!B40+SUM(MAX(C10*21*5-10000,0)/1000*2.83,MAX(C10*21*2-10000,0)/1000*5,MAX(C10*21*1-10000,0)/1000*5,MAX(C10*21*2-10000,0)/1000*5)*58</f>
+        <v/>
+      </c>
+      <c r="C10" s="8" t="n">
+        <v>5000</v>
+      </c>
+      <c r="D10" s="6">
+        <f>B10/C10</f>
         <v/>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>UI/UX and presentation support</t>
+          <t>City scale</t>
         </is>
       </c>
       <c r="B11" s="6">
-        <f>60000/1000000*Inputs!B37</f>
-        <v/>
-      </c>
-      <c r="C11" s="6">
-        <f>B11/6</f>
-        <v/>
-      </c>
-      <c r="D11" s="7">
-        <f>B11/SUM($B$5:$B$11)</f>
+        <f>Inputs!B40+SUM(MAX(C11*21*5-10000,0)/1000*2.83,MAX(C11*21*2-10000,0)/1000*5,MAX(C11*21*1-10000,0)/1000*5,MAX(C11*21*2-10000,0)/1000*5)*58</f>
+        <v/>
+      </c>
+      <c r="C11" s="8" t="n">
+        <v>10000</v>
+      </c>
+      <c r="D11" s="6">
+        <f>B11/C11</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="9" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
-      </c>
-      <c r="B12" s="9">
-        <f>SUM(B5:B11)</f>
-        <v/>
-      </c>
-      <c r="C12" s="9">
-        <f>SUM(C5:C11)</f>
-        <v/>
-      </c>
-      <c r="D12" s="9">
-        <f>SUM(D5:D11)</f>
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Metro scale stress test</t>
+        </is>
+      </c>
+      <c r="B12" s="6">
+        <f>Inputs!B40+SUM(MAX(C12*21*5-10000,0)/1000*2.83,MAX(C12*21*2-10000,0)/1000*5,MAX(C12*21*1-10000,0)/1000*5,MAX(C12*21*2-10000,0)/1000*5)*58</f>
+        <v/>
+      </c>
+      <c r="C12" s="8" t="n">
+        <v>25000</v>
+      </c>
+      <c r="D12" s="6">
+        <f>B12/C12</f>
         <v/>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -3170,16 +3555,234 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:D12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
+  <cols>
+    <col width="38" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="23.4" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Development Budget Allocation</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="n"/>
+      <c r="C1" s="2" t="n"/>
+      <c r="D1" s="2" t="n"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>Default allocation sums to PHP 1,000,000 and scales with the editable build budget.</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="n"/>
+      <c r="C2" s="2" t="n"/>
+      <c r="D2" s="2" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n"/>
+      <c r="B3" s="2" t="n"/>
+      <c r="C3" s="2" t="n"/>
+      <c r="D3" s="2" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Role</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>6-month allocation</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>Monthly allocation</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>Share</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Lead full-stack developer / PM</t>
+        </is>
+      </c>
+      <c r="B5" s="19">
+        <f>330000/1000000*Inputs!B37</f>
+        <v/>
+      </c>
+      <c r="C5" s="19">
+        <f>B5/6</f>
+        <v/>
+      </c>
+      <c r="D5" s="7">
+        <f>B5/SUM($B$5:$B$11)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Backend developer</t>
+        </is>
+      </c>
+      <c r="B6" s="19">
+        <f>180000/1000000*Inputs!B37</f>
+        <v/>
+      </c>
+      <c r="C6" s="19">
+        <f>B6/6</f>
+        <v/>
+      </c>
+      <c r="D6" s="7">
+        <f>B6/SUM($B$5:$B$11)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Frontend/mobile developer</t>
+        </is>
+      </c>
+      <c r="B7" s="19">
+        <f>140000/1000000*Inputs!B37</f>
+        <v/>
+      </c>
+      <c r="C7" s="19">
+        <f>B7/6</f>
+        <v/>
+      </c>
+      <c r="D7" s="7">
+        <f>B7/SUM($B$5:$B$11)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Cloud / DevOps engineer</t>
+        </is>
+      </c>
+      <c r="B8" s="19">
+        <f>120000/1000000*Inputs!B37</f>
+        <v/>
+      </c>
+      <c r="C8" s="19">
+        <f>B8/6</f>
+        <v/>
+      </c>
+      <c r="D8" s="7">
+        <f>B8/SUM($B$5:$B$11)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>QA and release support</t>
+        </is>
+      </c>
+      <c r="B9" s="19">
+        <f>90000/1000000*Inputs!B37</f>
+        <v/>
+      </c>
+      <c r="C9" s="19">
+        <f>B9/6</f>
+        <v/>
+      </c>
+      <c r="D9" s="7">
+        <f>B9/SUM($B$5:$B$11)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Product / client coordination</t>
+        </is>
+      </c>
+      <c r="B10" s="19">
+        <f>80000/1000000*Inputs!B37</f>
+        <v/>
+      </c>
+      <c r="C10" s="19">
+        <f>B10/6</f>
+        <v/>
+      </c>
+      <c r="D10" s="7">
+        <f>B10/SUM($B$5:$B$11)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>UI/UX and presentation support</t>
+        </is>
+      </c>
+      <c r="B11" s="19">
+        <f>60000/1000000*Inputs!B37</f>
+        <v/>
+      </c>
+      <c r="C11" s="19">
+        <f>B11/6</f>
+        <v/>
+      </c>
+      <c r="D11" s="7">
+        <f>B11/SUM($B$5:$B$11)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="9" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="B12" s="20">
+        <f>SUM(B5:B11)</f>
+        <v/>
+      </c>
+      <c r="C12" s="20">
+        <f>SUM(C5:C11)</f>
+        <v/>
+      </c>
+      <c r="D12" s="9">
+        <f>SUM(D5:D11)</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:B9"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
     <col width="90" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="3" max="4"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="23.4" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Model Notes</t>

</xml_diff>

<commit_message>
Correct cloud API tier costing
</commit_message>
<xml_diff>
--- a/eride_operating_model.xlsx
+++ b/eride_operating_model.xlsx
@@ -1284,7 +1284,7 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Recover AWS/cloud/API cost</t>
+          <t>Recover cloud/API cost</t>
         </is>
       </c>
       <c r="B7" s="5" t="n">
@@ -1297,7 +1297,7 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Includes workbook-based cloud/API scaling</t>
+          <t>Includes POC baseline plus Google Maps/Places/Routes API usage growth; full AWS production architecture should be priced separately</t>
         </is>
       </c>
     </row>
@@ -2287,7 +2287,7 @@
         <v/>
       </c>
       <c r="J6" s="17">
-        <f>((MIN(B6*D6,C6*E6*Inputs!B12)*Inputs!B13)*Model!B9*Inputs!B24 + B6*Inputs!B25) - (C6*Inputs!B26*Inputs!B12*(1+Inputs!B27) + C6*Inputs!B12*MAX(G6-Inputs!B28,0)*Inputs!B29 + (MIN(B6*D6,C6*E6*Inputs!B12)*Inputs!B13)*Inputs!B14*Inputs!B35*Inputs!B36 + IF(Inputs!B5=1,C6*(Inputs!B30+Inputs!B31)/Inputs!B32,0) + C6*(Inputs!B33+Inputs!B34) + IF(Inputs!B6=1,Inputs!B37/Inputs!B38+Inputs!B39,0) + IF(Inputs!B7=1,Inputs!B40+SUM(MAX(B6*21*5-10000,0)/1000*2.83,MAX(B6*21*2-10000,0)/1000*5,MAX(B6*21*1-10000,0)/1000*5,MAX(B6*21*2-10000,0)/1000*5)*58,0) + Inputs!B41+B6*(Inputs!B42+Inputs!B43) + ((MIN(B6*D6,C6*E6*Inputs!B12)*Inputs!B13)*Model!B9*Inputs!B24+B6*Inputs!B25)*Inputs!B44*Inputs!B45 + ((MIN(B6*D6,C6*E6*Inputs!B12)*Inputs!B13)*Model!B9*Inputs!B24+B6*Inputs!B25)*Inputs!B46)</f>
+        <f>((MIN(B6*D6,C6*E6*Inputs!B12)*Inputs!B13)*Model!B9*Inputs!B24 + B6*Inputs!B25) - (C6*Inputs!B26*Inputs!B12*(1+Inputs!B27) + C6*Inputs!B12*MAX(G6-Inputs!B28,0)*Inputs!B29 + (MIN(B6*D6,C6*E6*Inputs!B12)*Inputs!B13)*Inputs!B14*Inputs!B35*Inputs!B36 + IF(Inputs!B5=1,C6*(Inputs!B30+Inputs!B31)/Inputs!B32,0) + C6*(Inputs!B33+Inputs!B34) + IF(Inputs!B6=1,Inputs!B37/Inputs!B38+Inputs!B39,0) + IF(Inputs!B7=1,Inputs!B40+58*((MAX(MIN((B6)*Inputs!B12*5,100000)-10000,0))/1000*2.83+(MAX(MIN((B6)*Inputs!B12*5,500000)-100000,0))/1000*2.27+(MAX(MIN((B6)*Inputs!B12*5,1000000)-500000,0))/1000*1.7+(MAX(MIN((B6)*Inputs!B12*5,5000000)-1000000,0))/1000*0.85+(MAX((B6)*Inputs!B12*5-5000000,0))/1000*0.21+(MAX(MIN((B6)*Inputs!B12*2,100000)-10000,0))/1000*5+(MAX(MIN((B6)*Inputs!B12*2,500000)-100000,0))/1000*4+(MAX(MIN((B6)*Inputs!B12*2,1000000)-500000,0))/1000*3+(MAX(MIN((B6)*Inputs!B12*2,5000000)-1000000,0))/1000*1.5+(MAX((B6)*Inputs!B12*2-5000000,0))/1000*0.38+(MAX(MIN((B6)*Inputs!B12*1,100000)-10000,0))/1000*5+(MAX(MIN((B6)*Inputs!B12*1,500000)-100000,0))/1000*4+(MAX(MIN((B6)*Inputs!B12*1,1000000)-500000,0))/1000*3+(MAX(MIN((B6)*Inputs!B12*1,5000000)-1000000,0))/1000*1.5+(MAX((B6)*Inputs!B12*1-5000000,0))/1000*0.38+(MAX(MIN((B6)*Inputs!B12*2,100000)-10000,0))/1000*5+(MAX(MIN((B6)*Inputs!B12*2,500000)-100000,0))/1000*4+(MAX(MIN((B6)*Inputs!B12*2,1000000)-500000,0))/1000*3+(MAX(MIN((B6)*Inputs!B12*2,5000000)-1000000,0))/1000*1.5+(MAX((B6)*Inputs!B12*2-5000000,0))/1000*0.38),0) + Inputs!B41+B6*(Inputs!B42+Inputs!B43) + ((MIN(B6*D6,C6*E6*Inputs!B12)*Inputs!B13)*Model!B9*Inputs!B24+B6*Inputs!B25)*Inputs!B44*Inputs!B45 + ((MIN(B6*D6,C6*E6*Inputs!B12)*Inputs!B13)*Model!B9*Inputs!B24+B6*Inputs!B25)*Inputs!B46)</f>
         <v/>
       </c>
     </row>
@@ -2833,7 +2833,7 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>Cloud / API cost</t>
+          <t>Cloud/API usage cost</t>
         </is>
       </c>
       <c r="B27" s="6">
@@ -3335,7 +3335,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Cloud / API cost</t>
+          <t>Cloud/API usage cost</t>
         </is>
       </c>
       <c r="B12" s="6">
@@ -3440,7 +3440,7 @@
     <row r="1" ht="23.4" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>AWS / Cloud and API Cost Tiers</t>
+          <t>Cloud/API Cost Tiers</t>
         </is>
       </c>
       <c r="B1" s="2" t="n"/>
@@ -3450,7 +3450,7 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Uses the workbook-based Google Maps/API scaling plus POC baseline.</t>
+          <t>Uses workbook usage assumptions and official Google Maps Platform tiered pricing; AWS production architecture is not separately priced here.</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -3492,7 +3492,7 @@
         </is>
       </c>
       <c r="B5" s="6">
-        <f>Inputs!B40+SUM(MAX(C5*21*5-10000,0)/1000*2.83,MAX(C5*21*2-10000,0)/1000*5,MAX(C5*21*1-10000,0)/1000*5,MAX(C5*21*2-10000,0)/1000*5)*58</f>
+        <f>Inputs!B40+58*((MAX(MIN((C5)*Inputs!B12*5,100000)-10000,0))/1000*2.83+(MAX(MIN((C5)*Inputs!B12*5,500000)-100000,0))/1000*2.27+(MAX(MIN((C5)*Inputs!B12*5,1000000)-500000,0))/1000*1.7+(MAX(MIN((C5)*Inputs!B12*5,5000000)-1000000,0))/1000*0.85+(MAX((C5)*Inputs!B12*5-5000000,0))/1000*0.21+(MAX(MIN((C5)*Inputs!B12*2,100000)-10000,0))/1000*5+(MAX(MIN((C5)*Inputs!B12*2,500000)-100000,0))/1000*4+(MAX(MIN((C5)*Inputs!B12*2,1000000)-500000,0))/1000*3+(MAX(MIN((C5)*Inputs!B12*2,5000000)-1000000,0))/1000*1.5+(MAX((C5)*Inputs!B12*2-5000000,0))/1000*0.38+(MAX(MIN((C5)*Inputs!B12*1,100000)-10000,0))/1000*5+(MAX(MIN((C5)*Inputs!B12*1,500000)-100000,0))/1000*4+(MAX(MIN((C5)*Inputs!B12*1,1000000)-500000,0))/1000*3+(MAX(MIN((C5)*Inputs!B12*1,5000000)-1000000,0))/1000*1.5+(MAX((C5)*Inputs!B12*1-5000000,0))/1000*0.38+(MAX(MIN((C5)*Inputs!B12*2,100000)-10000,0))/1000*5+(MAX(MIN((C5)*Inputs!B12*2,500000)-100000,0))/1000*4+(MAX(MIN((C5)*Inputs!B12*2,1000000)-500000,0))/1000*3+(MAX(MIN((C5)*Inputs!B12*2,5000000)-1000000,0))/1000*1.5+(MAX((C5)*Inputs!B12*2-5000000,0))/1000*0.38)</f>
         <v/>
       </c>
       <c r="C5" s="8" t="n">
@@ -3510,7 +3510,7 @@
         </is>
       </c>
       <c r="B6" s="6">
-        <f>Inputs!B40+SUM(MAX(C6*21*5-10000,0)/1000*2.83,MAX(C6*21*2-10000,0)/1000*5,MAX(C6*21*1-10000,0)/1000*5,MAX(C6*21*2-10000,0)/1000*5)*58</f>
+        <f>Inputs!B40+58*((MAX(MIN((C6)*Inputs!B12*5,100000)-10000,0))/1000*2.83+(MAX(MIN((C6)*Inputs!B12*5,500000)-100000,0))/1000*2.27+(MAX(MIN((C6)*Inputs!B12*5,1000000)-500000,0))/1000*1.7+(MAX(MIN((C6)*Inputs!B12*5,5000000)-1000000,0))/1000*0.85+(MAX((C6)*Inputs!B12*5-5000000,0))/1000*0.21+(MAX(MIN((C6)*Inputs!B12*2,100000)-10000,0))/1000*5+(MAX(MIN((C6)*Inputs!B12*2,500000)-100000,0))/1000*4+(MAX(MIN((C6)*Inputs!B12*2,1000000)-500000,0))/1000*3+(MAX(MIN((C6)*Inputs!B12*2,5000000)-1000000,0))/1000*1.5+(MAX((C6)*Inputs!B12*2-5000000,0))/1000*0.38+(MAX(MIN((C6)*Inputs!B12*1,100000)-10000,0))/1000*5+(MAX(MIN((C6)*Inputs!B12*1,500000)-100000,0))/1000*4+(MAX(MIN((C6)*Inputs!B12*1,1000000)-500000,0))/1000*3+(MAX(MIN((C6)*Inputs!B12*1,5000000)-1000000,0))/1000*1.5+(MAX((C6)*Inputs!B12*1-5000000,0))/1000*0.38+(MAX(MIN((C6)*Inputs!B12*2,100000)-10000,0))/1000*5+(MAX(MIN((C6)*Inputs!B12*2,500000)-100000,0))/1000*4+(MAX(MIN((C6)*Inputs!B12*2,1000000)-500000,0))/1000*3+(MAX(MIN((C6)*Inputs!B12*2,5000000)-1000000,0))/1000*1.5+(MAX((C6)*Inputs!B12*2-5000000,0))/1000*0.38)</f>
         <v/>
       </c>
       <c r="C6" s="8" t="n">
@@ -3528,7 +3528,7 @@
         </is>
       </c>
       <c r="B7" s="6">
-        <f>Inputs!B40+SUM(MAX(C7*21*5-10000,0)/1000*2.83,MAX(C7*21*2-10000,0)/1000*5,MAX(C7*21*1-10000,0)/1000*5,MAX(C7*21*2-10000,0)/1000*5)*58</f>
+        <f>Inputs!B40+58*((MAX(MIN((C7)*Inputs!B12*5,100000)-10000,0))/1000*2.83+(MAX(MIN((C7)*Inputs!B12*5,500000)-100000,0))/1000*2.27+(MAX(MIN((C7)*Inputs!B12*5,1000000)-500000,0))/1000*1.7+(MAX(MIN((C7)*Inputs!B12*5,5000000)-1000000,0))/1000*0.85+(MAX((C7)*Inputs!B12*5-5000000,0))/1000*0.21+(MAX(MIN((C7)*Inputs!B12*2,100000)-10000,0))/1000*5+(MAX(MIN((C7)*Inputs!B12*2,500000)-100000,0))/1000*4+(MAX(MIN((C7)*Inputs!B12*2,1000000)-500000,0))/1000*3+(MAX(MIN((C7)*Inputs!B12*2,5000000)-1000000,0))/1000*1.5+(MAX((C7)*Inputs!B12*2-5000000,0))/1000*0.38+(MAX(MIN((C7)*Inputs!B12*1,100000)-10000,0))/1000*5+(MAX(MIN((C7)*Inputs!B12*1,500000)-100000,0))/1000*4+(MAX(MIN((C7)*Inputs!B12*1,1000000)-500000,0))/1000*3+(MAX(MIN((C7)*Inputs!B12*1,5000000)-1000000,0))/1000*1.5+(MAX((C7)*Inputs!B12*1-5000000,0))/1000*0.38+(MAX(MIN((C7)*Inputs!B12*2,100000)-10000,0))/1000*5+(MAX(MIN((C7)*Inputs!B12*2,500000)-100000,0))/1000*4+(MAX(MIN((C7)*Inputs!B12*2,1000000)-500000,0))/1000*3+(MAX(MIN((C7)*Inputs!B12*2,5000000)-1000000,0))/1000*1.5+(MAX((C7)*Inputs!B12*2-5000000,0))/1000*0.38)</f>
         <v/>
       </c>
       <c r="C7" s="8" t="n">
@@ -3546,7 +3546,7 @@
         </is>
       </c>
       <c r="B8" s="6">
-        <f>Inputs!B40+SUM(MAX(C8*21*5-10000,0)/1000*2.83,MAX(C8*21*2-10000,0)/1000*5,MAX(C8*21*1-10000,0)/1000*5,MAX(C8*21*2-10000,0)/1000*5)*58</f>
+        <f>Inputs!B40+58*((MAX(MIN((C8)*Inputs!B12*5,100000)-10000,0))/1000*2.83+(MAX(MIN((C8)*Inputs!B12*5,500000)-100000,0))/1000*2.27+(MAX(MIN((C8)*Inputs!B12*5,1000000)-500000,0))/1000*1.7+(MAX(MIN((C8)*Inputs!B12*5,5000000)-1000000,0))/1000*0.85+(MAX((C8)*Inputs!B12*5-5000000,0))/1000*0.21+(MAX(MIN((C8)*Inputs!B12*2,100000)-10000,0))/1000*5+(MAX(MIN((C8)*Inputs!B12*2,500000)-100000,0))/1000*4+(MAX(MIN((C8)*Inputs!B12*2,1000000)-500000,0))/1000*3+(MAX(MIN((C8)*Inputs!B12*2,5000000)-1000000,0))/1000*1.5+(MAX((C8)*Inputs!B12*2-5000000,0))/1000*0.38+(MAX(MIN((C8)*Inputs!B12*1,100000)-10000,0))/1000*5+(MAX(MIN((C8)*Inputs!B12*1,500000)-100000,0))/1000*4+(MAX(MIN((C8)*Inputs!B12*1,1000000)-500000,0))/1000*3+(MAX(MIN((C8)*Inputs!B12*1,5000000)-1000000,0))/1000*1.5+(MAX((C8)*Inputs!B12*1-5000000,0))/1000*0.38+(MAX(MIN((C8)*Inputs!B12*2,100000)-10000,0))/1000*5+(MAX(MIN((C8)*Inputs!B12*2,500000)-100000,0))/1000*4+(MAX(MIN((C8)*Inputs!B12*2,1000000)-500000,0))/1000*3+(MAX(MIN((C8)*Inputs!B12*2,5000000)-1000000,0))/1000*1.5+(MAX((C8)*Inputs!B12*2-5000000,0))/1000*0.38)</f>
         <v/>
       </c>
       <c r="C8" s="8" t="n">
@@ -3564,7 +3564,7 @@
         </is>
       </c>
       <c r="B9" s="6">
-        <f>Inputs!B40+SUM(MAX(C9*21*5-10000,0)/1000*2.83,MAX(C9*21*2-10000,0)/1000*5,MAX(C9*21*1-10000,0)/1000*5,MAX(C9*21*2-10000,0)/1000*5)*58</f>
+        <f>Inputs!B40+58*((MAX(MIN((C9)*Inputs!B12*5,100000)-10000,0))/1000*2.83+(MAX(MIN((C9)*Inputs!B12*5,500000)-100000,0))/1000*2.27+(MAX(MIN((C9)*Inputs!B12*5,1000000)-500000,0))/1000*1.7+(MAX(MIN((C9)*Inputs!B12*5,5000000)-1000000,0))/1000*0.85+(MAX((C9)*Inputs!B12*5-5000000,0))/1000*0.21+(MAX(MIN((C9)*Inputs!B12*2,100000)-10000,0))/1000*5+(MAX(MIN((C9)*Inputs!B12*2,500000)-100000,0))/1000*4+(MAX(MIN((C9)*Inputs!B12*2,1000000)-500000,0))/1000*3+(MAX(MIN((C9)*Inputs!B12*2,5000000)-1000000,0))/1000*1.5+(MAX((C9)*Inputs!B12*2-5000000,0))/1000*0.38+(MAX(MIN((C9)*Inputs!B12*1,100000)-10000,0))/1000*5+(MAX(MIN((C9)*Inputs!B12*1,500000)-100000,0))/1000*4+(MAX(MIN((C9)*Inputs!B12*1,1000000)-500000,0))/1000*3+(MAX(MIN((C9)*Inputs!B12*1,5000000)-1000000,0))/1000*1.5+(MAX((C9)*Inputs!B12*1-5000000,0))/1000*0.38+(MAX(MIN((C9)*Inputs!B12*2,100000)-10000,0))/1000*5+(MAX(MIN((C9)*Inputs!B12*2,500000)-100000,0))/1000*4+(MAX(MIN((C9)*Inputs!B12*2,1000000)-500000,0))/1000*3+(MAX(MIN((C9)*Inputs!B12*2,5000000)-1000000,0))/1000*1.5+(MAX((C9)*Inputs!B12*2-5000000,0))/1000*0.38)</f>
         <v/>
       </c>
       <c r="C9" s="8">
@@ -3583,7 +3583,7 @@
         </is>
       </c>
       <c r="B10" s="6">
-        <f>Inputs!B40+SUM(MAX(C10*21*5-10000,0)/1000*2.83,MAX(C10*21*2-10000,0)/1000*5,MAX(C10*21*1-10000,0)/1000*5,MAX(C10*21*2-10000,0)/1000*5)*58</f>
+        <f>Inputs!B40+58*((MAX(MIN((C10)*Inputs!B12*5,100000)-10000,0))/1000*2.83+(MAX(MIN((C10)*Inputs!B12*5,500000)-100000,0))/1000*2.27+(MAX(MIN((C10)*Inputs!B12*5,1000000)-500000,0))/1000*1.7+(MAX(MIN((C10)*Inputs!B12*5,5000000)-1000000,0))/1000*0.85+(MAX((C10)*Inputs!B12*5-5000000,0))/1000*0.21+(MAX(MIN((C10)*Inputs!B12*2,100000)-10000,0))/1000*5+(MAX(MIN((C10)*Inputs!B12*2,500000)-100000,0))/1000*4+(MAX(MIN((C10)*Inputs!B12*2,1000000)-500000,0))/1000*3+(MAX(MIN((C10)*Inputs!B12*2,5000000)-1000000,0))/1000*1.5+(MAX((C10)*Inputs!B12*2-5000000,0))/1000*0.38+(MAX(MIN((C10)*Inputs!B12*1,100000)-10000,0))/1000*5+(MAX(MIN((C10)*Inputs!B12*1,500000)-100000,0))/1000*4+(MAX(MIN((C10)*Inputs!B12*1,1000000)-500000,0))/1000*3+(MAX(MIN((C10)*Inputs!B12*1,5000000)-1000000,0))/1000*1.5+(MAX((C10)*Inputs!B12*1-5000000,0))/1000*0.38+(MAX(MIN((C10)*Inputs!B12*2,100000)-10000,0))/1000*5+(MAX(MIN((C10)*Inputs!B12*2,500000)-100000,0))/1000*4+(MAX(MIN((C10)*Inputs!B12*2,1000000)-500000,0))/1000*3+(MAX(MIN((C10)*Inputs!B12*2,5000000)-1000000,0))/1000*1.5+(MAX((C10)*Inputs!B12*2-5000000,0))/1000*0.38)</f>
         <v/>
       </c>
       <c r="C10" s="8" t="n">
@@ -3601,7 +3601,7 @@
         </is>
       </c>
       <c r="B11" s="6">
-        <f>Inputs!B40+SUM(MAX(C11*21*5-10000,0)/1000*2.83,MAX(C11*21*2-10000,0)/1000*5,MAX(C11*21*1-10000,0)/1000*5,MAX(C11*21*2-10000,0)/1000*5)*58</f>
+        <f>Inputs!B40+58*((MAX(MIN((C11)*Inputs!B12*5,100000)-10000,0))/1000*2.83+(MAX(MIN((C11)*Inputs!B12*5,500000)-100000,0))/1000*2.27+(MAX(MIN((C11)*Inputs!B12*5,1000000)-500000,0))/1000*1.7+(MAX(MIN((C11)*Inputs!B12*5,5000000)-1000000,0))/1000*0.85+(MAX((C11)*Inputs!B12*5-5000000,0))/1000*0.21+(MAX(MIN((C11)*Inputs!B12*2,100000)-10000,0))/1000*5+(MAX(MIN((C11)*Inputs!B12*2,500000)-100000,0))/1000*4+(MAX(MIN((C11)*Inputs!B12*2,1000000)-500000,0))/1000*3+(MAX(MIN((C11)*Inputs!B12*2,5000000)-1000000,0))/1000*1.5+(MAX((C11)*Inputs!B12*2-5000000,0))/1000*0.38+(MAX(MIN((C11)*Inputs!B12*1,100000)-10000,0))/1000*5+(MAX(MIN((C11)*Inputs!B12*1,500000)-100000,0))/1000*4+(MAX(MIN((C11)*Inputs!B12*1,1000000)-500000,0))/1000*3+(MAX(MIN((C11)*Inputs!B12*1,5000000)-1000000,0))/1000*1.5+(MAX((C11)*Inputs!B12*1-5000000,0))/1000*0.38+(MAX(MIN((C11)*Inputs!B12*2,100000)-10000,0))/1000*5+(MAX(MIN((C11)*Inputs!B12*2,500000)-100000,0))/1000*4+(MAX(MIN((C11)*Inputs!B12*2,1000000)-500000,0))/1000*3+(MAX(MIN((C11)*Inputs!B12*2,5000000)-1000000,0))/1000*1.5+(MAX((C11)*Inputs!B12*2-5000000,0))/1000*0.38)</f>
         <v/>
       </c>
       <c r="C11" s="8" t="n">
@@ -3619,7 +3619,7 @@
         </is>
       </c>
       <c r="B12" s="6">
-        <f>Inputs!B40+SUM(MAX(C12*21*5-10000,0)/1000*2.83,MAX(C12*21*2-10000,0)/1000*5,MAX(C12*21*1-10000,0)/1000*5,MAX(C12*21*2-10000,0)/1000*5)*58</f>
+        <f>Inputs!B40+58*((MAX(MIN((C12)*Inputs!B12*5,100000)-10000,0))/1000*2.83+(MAX(MIN((C12)*Inputs!B12*5,500000)-100000,0))/1000*2.27+(MAX(MIN((C12)*Inputs!B12*5,1000000)-500000,0))/1000*1.7+(MAX(MIN((C12)*Inputs!B12*5,5000000)-1000000,0))/1000*0.85+(MAX((C12)*Inputs!B12*5-5000000,0))/1000*0.21+(MAX(MIN((C12)*Inputs!B12*2,100000)-10000,0))/1000*5+(MAX(MIN((C12)*Inputs!B12*2,500000)-100000,0))/1000*4+(MAX(MIN((C12)*Inputs!B12*2,1000000)-500000,0))/1000*3+(MAX(MIN((C12)*Inputs!B12*2,5000000)-1000000,0))/1000*1.5+(MAX((C12)*Inputs!B12*2-5000000,0))/1000*0.38+(MAX(MIN((C12)*Inputs!B12*1,100000)-10000,0))/1000*5+(MAX(MIN((C12)*Inputs!B12*1,500000)-100000,0))/1000*4+(MAX(MIN((C12)*Inputs!B12*1,1000000)-500000,0))/1000*3+(MAX(MIN((C12)*Inputs!B12*1,5000000)-1000000,0))/1000*1.5+(MAX((C12)*Inputs!B12*1-5000000,0))/1000*0.38+(MAX(MIN((C12)*Inputs!B12*2,100000)-10000,0))/1000*5+(MAX(MIN((C12)*Inputs!B12*2,500000)-100000,0))/1000*4+(MAX(MIN((C12)*Inputs!B12*2,1000000)-500000,0))/1000*3+(MAX(MIN((C12)*Inputs!B12*2,5000000)-1000000,0))/1000*1.5+(MAX((C12)*Inputs!B12*2-5000000,0))/1000*0.38)</f>
         <v/>
       </c>
       <c r="C12" s="8" t="n">
@@ -3949,7 +3949,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>POC baseline is PHP 1,500. Growth uses 21 days, PHP 58/USD, 10,000 free monthly events per priced API, and per-user daily API ratios from the Dev Costing Foundation workbook.</t>
+          <t>Cloud/API tiers use PHP 58/USD, operating days/month from Inputs, workbook usage ratios, and official Google Maps Platform tiered pricing. AWS production server/database/storage architecture is not separately priced here.</t>
         </is>
       </c>
     </row>

</xml_diff>